<commit_message>
هبوط 2US100 30 OC-21-NOV
</commit_message>
<xml_diff>
--- a/docs/اختبار المتوسطه.xlsx
+++ b/docs/اختبار المتوسطه.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\MA-Waves\MA-Waves\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85218EA8-C6DF-4AF2-BBBF-55806F1BB8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F640878A-8FF0-4F5C-9EE0-7D767ED79C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{7819BD92-4B63-487D-A2E5-7EFEA3C3CD0C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{7819BD92-4B63-487D-A2E5-7EFEA3C3CD0C}"/>
   </bookViews>
   <sheets>
     <sheet name="هبوط" sheetId="3" r:id="rId1"/>
     <sheet name="صعود" sheetId="2" r:id="rId2"/>
     <sheet name="صعود 2 " sheetId="1" r:id="rId3"/>
+    <sheet name="هبوط 2US100 30 OC-21-NOV " sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="64">
   <si>
     <t>#</t>
   </si>
@@ -86,6 +87,9 @@
     <t>قاع صغيره</t>
   </si>
   <si>
+    <t>قمه</t>
+  </si>
+  <si>
     <t>قمه صغير</t>
   </si>
   <si>
@@ -189,6 +193,33 @@
   </si>
   <si>
     <t>قاع صغير : المتوقع قاع متوسط لانه القاع الذي بعد الكسر</t>
+  </si>
+  <si>
+    <t>متوسطه</t>
+  </si>
+  <si>
+    <t>صغير</t>
+  </si>
+  <si>
+    <t>يجب ان يمسع بقانون الفعاليه</t>
+  </si>
+  <si>
+    <t>يجب ان يمسح بقانون التتابع</t>
+  </si>
+  <si>
+    <t>صحيح</t>
+  </si>
+  <si>
+    <t>سحيح</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رسم ك متوسط وهذا خاطئ لم يحدث كسر </t>
+  </si>
+  <si>
+    <t>رسم ك صغير يجب ان يكون متوسط لانه القاع الذي سبق الكسر</t>
+  </si>
+  <si>
+    <t>رسم ك صغير يجب ان يكون متوسط لانه القمه التي بعد الكسر</t>
   </si>
 </sst>
 </file>
@@ -694,7 +725,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -709,10 +740,10 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -729,13 +760,13 @@
         <v>6</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -773,10 +804,10 @@
         <v>9</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G4" s="4"/>
     </row>
@@ -815,10 +846,10 @@
         <v>10</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G6" s="4"/>
     </row>
@@ -836,13 +867,13 @@
         <v>8</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -859,13 +890,13 @@
         <v>9</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -903,13 +934,13 @@
         <v>9</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -947,10 +978,10 @@
         <v>9</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G12" s="4"/>
     </row>
@@ -971,10 +1002,10 @@
         <v>15</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -991,13 +1022,13 @@
         <v>9</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1035,13 +1066,13 @@
         <v>11</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1079,10 +1110,10 @@
         <v>9</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G18" s="4"/>
     </row>
@@ -1121,10 +1152,10 @@
         <v>9</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G20" s="4"/>
     </row>
@@ -1145,10 +1176,10 @@
         <v>16</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1165,13 +1196,13 @@
         <v>13</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -1191,10 +1222,10 @@
         <v>16</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1211,13 +1242,13 @@
         <v>11</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1255,10 +1286,10 @@
         <v>11</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G26" s="4"/>
     </row>
@@ -1297,10 +1328,10 @@
         <v>12</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G28" s="4"/>
     </row>
@@ -1337,10 +1368,10 @@
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G30" s="4"/>
     </row>
@@ -1365,7 +1396,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -1383,7 +1414,7 @@
         <v>14</v>
       </c>
       <c r="G1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1397,16 +1428,16 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1423,10 +1454,10 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1440,7 +1471,7 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
         <v>16</v>
@@ -1480,7 +1511,7 @@
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" t="s">
         <v>16</v>
@@ -1520,7 +1551,7 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E8" t="s">
         <v>16</v>
@@ -1543,13 +1574,13 @@
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1563,16 +1594,16 @@
         <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E10" t="s">
         <v>16</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1586,16 +1617,16 @@
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1609,7 +1640,7 @@
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
         <v>18</v>
@@ -1632,13 +1663,13 @@
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1652,16 +1683,16 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E14" t="s">
         <v>18</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1675,16 +1706,16 @@
         <v>5</v>
       </c>
       <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" t="s">
         <v>29</v>
-      </c>
-      <c r="E15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F15" t="s">
-        <v>20</v>
-      </c>
-      <c r="G15" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1698,16 +1729,16 @@
         <v>7</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1741,7 +1772,7 @@
         <v>7</v>
       </c>
       <c r="D18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E18" t="s">
         <v>18</v>
@@ -1764,10 +1795,10 @@
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1781,7 +1812,7 @@
         <v>7</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E20" s="12" t="s">
         <v>18</v>
@@ -1804,10 +1835,10 @@
         <v>11</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1844,7 +1875,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1862,12 +1893,12 @@
         <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
@@ -1891,7 +1922,7 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -2028,16 +2059,16 @@
         <v>5</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -2054,13 +2085,13 @@
         <v>7</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2077,7 +2108,7 @@
         <v>5</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F12" t="s">
         <v>17</v>
@@ -2117,10 +2148,10 @@
         <v>5</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -2140,7 +2171,7 @@
         <v>16</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -2157,16 +2188,16 @@
         <v>5</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -2183,7 +2214,7 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -2234,7 +2265,7 @@
         <v>5</v>
       </c>
       <c r="E20" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -2317,4 +2348,325 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A0CEE51-D789-43A5-978F-DA5C37A88868}">
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="39.85546875" customWidth="1"/>
+    <col min="5" max="5" width="46" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11">
+        <v>26259.29</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11">
+        <v>25713.11</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11">
+        <v>26136.6</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11">
+        <v>25166.29</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11">
+        <v>25427.040000000001</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11">
+        <v>25284.85</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>5</v>
+      </c>
+      <c r="B8" s="11">
+        <v>25759.49</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>6</v>
+      </c>
+      <c r="B9" s="11">
+        <v>25053.4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>7</v>
+      </c>
+      <c r="B10" s="11">
+        <v>25242.19</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>8</v>
+      </c>
+      <c r="B11" s="11">
+        <v>24611.87</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>9</v>
+      </c>
+      <c r="B12" s="11">
+        <v>25676.959999999999</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>10</v>
+      </c>
+      <c r="B13" s="11">
+        <v>25389.34</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>11</v>
+      </c>
+      <c r="B14" s="11">
+        <v>25727.59</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>12</v>
+      </c>
+      <c r="B15" s="11">
+        <v>24536.68</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>13</v>
+      </c>
+      <c r="B16" s="11">
+        <v>25269.98</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>14</v>
+      </c>
+      <c r="B17" s="11">
+        <v>24306.46</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>15</v>
+      </c>
+      <c r="B18" s="11">
+        <v>25219.98</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>